<commit_message>
more than one normality checks added
</commit_message>
<xml_diff>
--- a/logs/massive_topology_search/massive_topology_search.xlsx
+++ b/logs/massive_topology_search/massive_topology_search.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mgep-my.sharepoint.com/personal/uxue_ballarin_alumni_mondragon_edu/Documents/Semestre 8-Erasmus/Simula/ship_qnn/logs/massive_topology_search/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="219" documentId="11_AD4D2F04E46CFB4ACB3E20D455D6CCDA693EDF1F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EC38DEB0-993A-4CB1-89CD-BFFD4B9E3197}"/>
+  <xr:revisionPtr revIDLastSave="232" documentId="11_AD4D2F04E46CFB4ACB3E20D455D6CCDA693EDF1F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{006836B1-E337-4C38-8D4B-52908CCEF2AD}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2370" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2446" uniqueCount="272">
   <si>
     <t>date</t>
   </si>
@@ -831,6 +831,21 @@
   <si>
     <t>03-03_07-18-06_multihead_spsa_compact_f5_w5_h5_effsu2_lin_r2.pkl</t>
   </si>
+  <si>
+    <t>03-03_13-50-32_multihead_spsa_compact_f5_w5_h5_effsu2_lin_r2.pkl</t>
+  </si>
+  <si>
+    <t>03-03_21-45-50_multihead_spsa_compact_f5_w5_h5_effsu2_lin_r3.pkl</t>
+  </si>
+  <si>
+    <t>[{'features': ['wv', 'rarad'], 'output_dim': 1, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 1, -1]}, {'features': ['sv', 'rarad'], 'output_dim': 1, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 1, -1]}, {'features': ['yr', 'rarad'], 'output_dim': 1, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 1, -1]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 1, -1]}]</t>
+  </si>
+  <si>
+    <t>03-04_05-20-44_multihead_spsa_compact_f5_w5_h5_effsu2_lin_r3.pkl</t>
+  </si>
+  <si>
+    <t>03-04_13-32-28_multihead_spsa_compact_f5_w5_h5_effsu2_lin_r3.pkl</t>
+  </si>
 </sst>
 </file>
 
@@ -973,13 +988,13 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Uxue Ballarin" refreshedDate="46084.590416203704" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="116" xr:uid="{74ED0919-17AD-467A-B408-AADD8AC7697B}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Uxue Ballarin" refreshedDate="46086.568596759258" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="120" xr:uid="{74ED0919-17AD-467A-B408-AADD8AC7697B}">
   <cacheSource type="worksheet">
     <worksheetSource name="Tabla1"/>
   </cacheSource>
   <cacheFields count="75">
     <cacheField name="date" numFmtId="164">
-      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2026-02-17T13:56:47" maxDate="2026-03-03T07:18:06"/>
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2026-02-17T13:56:47" maxDate="2026-03-04T13:32:28"/>
     </cacheField>
     <cacheField name="model_id" numFmtId="0">
       <sharedItems/>
@@ -1190,25 +1205,25 @@
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="-1.9508774442032091" maxValue="0.759048124160834"/>
     </cacheField>
     <cacheField name="Yaw Rate Step MSE" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="3.7365891845960029E-2" maxValue="0.2321027489969984"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="2.8422902017742321E-2" maxValue="0.2321027489969984"/>
     </cacheField>
     <cacheField name="Yaw Rate Step R2" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="6.8180877318678279E-2" maxValue="0.84998776314123747"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="6.8180877318678279E-2" maxValue="0.88589103861681395"/>
     </cacheField>
     <cacheField name="Yaw Rate Local MSE" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="3.7365891845960029E-2" maxValue="0.2321027489969984"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="2.8422902017742321E-2" maxValue="0.2321027489969984"/>
     </cacheField>
     <cacheField name="Yaw Rate Global open MSE" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="3.7365891845960029E-2" maxValue="0.2321027489969984"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="2.8422902017742321E-2" maxValue="0.2321027489969984"/>
     </cacheField>
     <cacheField name="Yaw Rate Global open R2" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="6.8180877318678279E-2" maxValue="0.84998776314123747"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="6.8180877318678279E-2" maxValue="0.88589103861681395"/>
     </cacheField>
     <cacheField name="Yaw Rate Global closed MSE" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="7.6995679521455779E-2" maxValue="0.47455718790751072"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="7.2238055104180895E-2" maxValue="0.80870605181118038"/>
     </cacheField>
     <cacheField name="Yaw Rate Global closed R2" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="-0.90519700610616405" maxValue="0.69088670060145219"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="-2.2466990027572451" maxValue="0.70998705779114513"/>
     </cacheField>
     <cacheField name="Yaw Angle Step MSE" numFmtId="0">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="20.09951675360124" maxValue="205.0599827949176"/>
@@ -1241,7 +1256,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="116">
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="120">
   <r>
     <d v="2026-02-22T09:16:08"/>
     <s v="02-22_09-16-08_multihead_spsa_compact_f5_w5_h5_effsu2_effsu2_realamplitudes_lin_r1_3_1.pkl"/>
@@ -10174,12 +10189,320 @@
     <n v="350.38007034092919"/>
     <n v="2.75655493797955E-3"/>
   </r>
+  <r>
+    <d v="2026-03-03T13:50:32"/>
+    <s v="03-03_13-50-32_multihead_spsa_compact_f5_w5_h5_effsu2_lin_r2.pkl"/>
+    <x v="2"/>
+    <s v="Final (Last Iteration)"/>
+    <s v="data/reduce_row_number_absolutes"/>
+    <n v="16590"/>
+    <n v="4.5"/>
+    <s v="[['wv', 'rarad'], ['sv', 'rarad'], ['yr', 'rarad'], ['ya', 'yr']]"/>
+    <s v="['Surge Velocity', 'Sway Velocity', 'Yaw Rate', 'Yaw Angle']"/>
+    <n v="5"/>
+    <n v="5"/>
+    <s v="motion"/>
+    <s v="true"/>
+    <s v="false"/>
+    <s v="false"/>
+    <s v="multihead"/>
+    <s v="[{'features': ['wv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 1, -1]}, {'features': ['sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 1, -1]}, {'features': ['yr', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 1, -1]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 1, -1]}]"/>
+    <x v="1"/>
+    <s v="compact"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="5"/>
+    <s v="[0, 1, -1]"/>
+    <s v="false"/>
+    <s v="spsa"/>
+    <n v="4000"/>
+    <n v="4000"/>
+    <m/>
+    <n v="512"/>
+    <s v="[0.05, 0.001]"/>
+    <n v="0.1"/>
+    <n v="200"/>
+    <n v="80"/>
+    <n v="120"/>
+    <n v="8.1052205736362792E-2"/>
+    <n v="14.22849995965816"/>
+    <n v="0.77746501612623886"/>
+    <n v="-0.3388975246539947"/>
+    <n v="15.862007738386041"/>
+    <n v="0.78442861878483838"/>
+    <n v="15.862007738386041"/>
+    <n v="15.862007738386041"/>
+    <n v="0.78442861878483838"/>
+    <n v="121.20113997537661"/>
+    <n v="-8.1210961546633792E-2"/>
+    <n v="0.8"/>
+    <s v="identity"/>
+    <n v="2.8301968546252301E-2"/>
+    <n v="0.79449111508239822"/>
+    <n v="2.8301968546252301E-2"/>
+    <n v="2.8301968546252301E-2"/>
+    <n v="0.79449111508239822"/>
+    <n v="8.7375441623793029E-2"/>
+    <n v="0.36554132098820119"/>
+    <n v="8.5353100083140371E-2"/>
+    <n v="0.70426973809866467"/>
+    <n v="8.5353100083140371E-2"/>
+    <n v="8.5353100083140371E-2"/>
+    <n v="0.70426973809866467"/>
+    <n v="0.25345929775810411"/>
+    <n v="0.12181766761464741"/>
+    <n v="4.5063036259409023E-2"/>
+    <n v="0.81908616294267955"/>
+    <n v="4.5063036259409023E-2"/>
+    <n v="4.5063036259409023E-2"/>
+    <n v="0.81908616294267955"/>
+    <n v="0.35727610205897897"/>
+    <n v="-0.43435054265516498"/>
+    <n v="63.289312848655371"/>
+    <n v="0.81986745901560942"/>
+    <n v="63.289312848655371"/>
+    <n v="63.289312848655371"/>
+    <n v="0.81986745901560942"/>
+    <n v="484.10644906006519"/>
+    <n v="-0.37785229213422711"/>
+  </r>
+  <r>
+    <d v="2026-03-03T21:45:50"/>
+    <s v="03-03_21-45-50_multihead_spsa_compact_f5_w5_h5_effsu2_lin_r3.pkl"/>
+    <x v="1"/>
+    <s v="Final (Last Iteration)"/>
+    <s v="data/reduce_row_number_absolutes"/>
+    <n v="16590"/>
+    <n v="4.5"/>
+    <s v="[['wv', 'rarad'], ['sv', 'rarad'], ['yr', 'rarad'], ['ya', 'yr']]"/>
+    <s v="['Surge Velocity', 'Sway Velocity', 'Yaw Rate', 'Yaw Angle']"/>
+    <n v="5"/>
+    <n v="5"/>
+    <s v="motion"/>
+    <s v="true"/>
+    <s v="false"/>
+    <s v="false"/>
+    <s v="multihead"/>
+    <s v="[{'features': ['wv', 'rarad'], 'output_dim': 1, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 1, -1]}, {'features': ['sv', 'rarad'], 'output_dim': 1, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 1, -1]}, {'features': ['yr', 'rarad'], 'output_dim': 1, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 1, -1]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 1, -1]}]"/>
+    <x v="1"/>
+    <s v="compact"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="2"/>
+    <s v="[0, 1, -1]"/>
+    <s v="false"/>
+    <s v="spsa"/>
+    <n v="4000"/>
+    <n v="4000"/>
+    <m/>
+    <n v="512"/>
+    <s v="[0.05, 0.001]"/>
+    <n v="0.1"/>
+    <n v="240"/>
+    <n v="120"/>
+    <n v="120"/>
+    <n v="0.106008494446163"/>
+    <n v="33.838931129888543"/>
+    <n v="0.66621549860948348"/>
+    <n v="5.3792376803492359E-2"/>
+    <n v="35.082387455197612"/>
+    <n v="0.68480606442805336"/>
+    <n v="35.082387455197612"/>
+    <n v="35.082387455197612"/>
+    <n v="0.68480606442805336"/>
+    <n v="114.439596298278"/>
+    <n v="-0.61720424299988363"/>
+    <n v="0.8"/>
+    <s v="identity"/>
+    <n v="3.8320129051456348E-2"/>
+    <n v="0.72174631674847922"/>
+    <n v="3.8320129051456348E-2"/>
+    <n v="3.8320129051456348E-2"/>
+    <n v="0.72174631674847922"/>
+    <n v="0.1118626898969249"/>
+    <n v="0.1877322375285925"/>
+    <n v="8.0002391425953584E-2"/>
+    <n v="0.72280880078070253"/>
+    <n v="8.0002391425953584E-2"/>
+    <n v="8.0002391425953584E-2"/>
+    <n v="0.72280880078070253"/>
+    <n v="0.3205165810134426"/>
+    <n v="-0.1105214966357024"/>
+    <n v="7.6340327560767682E-2"/>
+    <n v="0.69351773143454143"/>
+    <n v="7.6340327560767682E-2"/>
+    <n v="7.6340327560767682E-2"/>
+    <n v="0.69351773143454143"/>
+    <n v="0.80870605181118038"/>
+    <n v="-2.2466990027572451"/>
+    <n v="140.13488697275301"/>
+    <n v="0.6011514087484886"/>
+    <n v="140.13488697275301"/>
+    <n v="140.13488697275301"/>
+    <n v="0.6011514087484886"/>
+    <n v="456.51729987039209"/>
+    <n v="-0.29932871013520312"/>
+  </r>
+  <r>
+    <d v="2026-03-04T05:20:44"/>
+    <s v="03-04_05-20-44_multihead_spsa_compact_f5_w5_h5_effsu2_lin_r3.pkl"/>
+    <x v="0"/>
+    <s v="Final (Last Iteration)"/>
+    <s v="data/reduce_row_number_absolutes"/>
+    <n v="16590"/>
+    <n v="4.5"/>
+    <s v="[['wv', 'rarad'], ['sv', 'rarad'], ['yr', 'rarad'], ['ya', 'yr']]"/>
+    <s v="['Surge Velocity', 'Sway Velocity', 'Yaw Rate', 'Yaw Angle']"/>
+    <n v="5"/>
+    <n v="5"/>
+    <s v="motion"/>
+    <s v="true"/>
+    <s v="false"/>
+    <s v="false"/>
+    <s v="multihead"/>
+    <s v="[{'features': ['wv', 'rarad'], 'output_dim': 1, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 1, -1]}, {'features': ['sv', 'rarad'], 'output_dim': 1, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 1, -1]}, {'features': ['yr', 'rarad'], 'output_dim': 1, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 1, -1]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 1, -1]}]"/>
+    <x v="1"/>
+    <s v="compact"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="2"/>
+    <s v="[0, 1, -1]"/>
+    <s v="false"/>
+    <s v="spsa"/>
+    <n v="4000"/>
+    <n v="4000"/>
+    <m/>
+    <n v="512"/>
+    <s v="[0.05, 0.001]"/>
+    <n v="0.1"/>
+    <n v="240"/>
+    <n v="120"/>
+    <n v="120"/>
+    <n v="8.6326044526204557E-2"/>
+    <n v="14.146799722733681"/>
+    <n v="0.72262530601792541"/>
+    <n v="7.581434566459494E-2"/>
+    <n v="25.026228384313718"/>
+    <n v="0.73291761438861314"/>
+    <n v="25.026228384313718"/>
+    <n v="25.026228384313718"/>
+    <n v="0.73291761438861314"/>
+    <n v="120.5007286916416"/>
+    <n v="4.6809187335239033E-2"/>
+    <n v="0.8"/>
+    <s v="identity"/>
+    <n v="4.3604468438270379E-2"/>
+    <n v="0.68337518036849354"/>
+    <n v="4.3604468438270379E-2"/>
+    <n v="4.3604468438270379E-2"/>
+    <n v="0.68337518036849354"/>
+    <n v="0.15250768795884201"/>
+    <n v="-0.10740300069810479"/>
+    <n v="0.10193258953106291"/>
+    <n v="0.64682534824230808"/>
+    <n v="0.10193258953106291"/>
+    <n v="0.10193258953106291"/>
+    <n v="0.64682534824230808"/>
+    <n v="0.30160015428650921"/>
+    <n v="-4.4980118235335993E-2"/>
+    <n v="2.8422902017742321E-2"/>
+    <n v="0.88589103861681395"/>
+    <n v="2.8422902017742321E-2"/>
+    <n v="2.8422902017742321E-2"/>
+    <n v="0.88589103861681395"/>
+    <n v="7.2238055104180895E-2"/>
+    <n v="0.70998705779114513"/>
+    <n v="99.930953577267957"/>
+    <n v="0.7155788903268383"/>
+    <n v="99.930953577267957"/>
+    <n v="99.930953577267957"/>
+    <n v="0.7155788903268383"/>
+    <n v="481.47656886921482"/>
+    <n v="-0.37036718951674041"/>
+  </r>
+  <r>
+    <d v="2026-03-04T13:32:28"/>
+    <s v="03-04_13-32-28_multihead_spsa_compact_f5_w5_h5_effsu2_lin_r3.pkl"/>
+    <x v="2"/>
+    <s v="Best (Lowest Val Loss)"/>
+    <s v="data/reduce_row_number_absolutes"/>
+    <n v="16590"/>
+    <n v="4.5"/>
+    <s v="[['wv', 'rarad'], ['sv', 'rarad'], ['yr', 'rarad'], ['ya', 'yr']]"/>
+    <s v="['Surge Velocity', 'Sway Velocity', 'Yaw Rate', 'Yaw Angle']"/>
+    <n v="5"/>
+    <n v="5"/>
+    <s v="motion"/>
+    <s v="true"/>
+    <s v="false"/>
+    <s v="false"/>
+    <s v="multihead"/>
+    <s v="[{'features': ['wv', 'rarad'], 'output_dim': 1, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 1, -1]}, {'features': ['sv', 'rarad'], 'output_dim': 1, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 1, -1]}, {'features': ['yr', 'rarad'], 'output_dim': 1, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 1, -1]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 1, -1]}]"/>
+    <x v="1"/>
+    <s v="compact"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="2"/>
+    <s v="[0, 1, -1]"/>
+    <s v="false"/>
+    <s v="spsa"/>
+    <n v="4000"/>
+    <n v="4000"/>
+    <m/>
+    <n v="512"/>
+    <s v="[0.05, 0.001]"/>
+    <n v="0.1"/>
+    <n v="240"/>
+    <n v="120"/>
+    <n v="120"/>
+    <n v="0.10290996228240711"/>
+    <n v="26.931966029656579"/>
+    <n v="0.68443970848741087"/>
+    <n v="8.6293657915927025E-2"/>
+    <n v="28.812146797667111"/>
+    <n v="0.67734594458609443"/>
+    <n v="28.812146797667111"/>
+    <n v="28.812146797667111"/>
+    <n v="0.67734594458609443"/>
+    <n v="112.7319246644321"/>
+    <n v="1.2595647239736749E-2"/>
+    <n v="0.8"/>
+    <s v="identity"/>
+    <n v="3.4941550989431677E-2"/>
+    <n v="0.74627916184012233"/>
+    <n v="3.4941550989431677E-2"/>
+    <n v="3.4941550989431677E-2"/>
+    <n v="0.74627916184012233"/>
+    <n v="0.1223043357798201"/>
+    <n v="0.1119123878036022"/>
+    <n v="0.1088797158354875"/>
+    <n v="0.62275503937868226"/>
+    <n v="0.1088797158354875"/>
+    <n v="0.1088797158354875"/>
+    <n v="0.62275503937868226"/>
+    <n v="0.26707186033242392"/>
+    <n v="7.465304569311626E-2"/>
+    <n v="8.2765557334563297E-2"/>
+    <n v="0.66772246620516862"/>
+    <n v="8.2765557334563297E-2"/>
+    <n v="8.2765557334563297E-2"/>
+    <n v="0.66772246620516862"/>
+    <n v="0.21283797098879029"/>
+    <n v="0.14552286753565319"/>
+    <n v="115.0220003665092"/>
+    <n v="0.6726271109204025"/>
+    <n v="115.0220003665092"/>
+    <n v="115.0220003665092"/>
+    <n v="0.6726271109204025"/>
+    <n v="450.32548449062648"/>
+    <n v="-0.28170571207342049"/>
+  </r>
 </pivotCacheRecords>
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2D21AEEF-8491-4048-847C-B48B541C6815}" name="TablaDinámica1" cacheId="24" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A2:L67" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A2:L68" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="75">
     <pivotField numFmtId="164" showAll="0"/>
     <pivotField dataField="1" showAll="0"/>
@@ -10307,7 +10630,7 @@
     <field x="21"/>
     <field x="2"/>
   </rowFields>
-  <rowItems count="65">
+  <rowItems count="66">
     <i>
       <x/>
     </i>
@@ -10498,6 +10821,9 @@
       <x v="1"/>
     </i>
     <i r="3">
+      <x/>
+    </i>
+    <i r="3">
       <x v="6"/>
     </i>
     <i t="grand">
@@ -10568,8 +10894,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3111F1FF-B489-4444-B033-EAAA6A990F8A}" name="Tabla1" displayName="Tabla1" ref="A1:BW117" totalsRowShown="0" headerRowDxfId="3" headerRowBorderDxfId="2" tableBorderDxfId="1">
-  <autoFilter ref="A1:BW117" xr:uid="{3111F1FF-B489-4444-B033-EAAA6A990F8A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3111F1FF-B489-4444-B033-EAAA6A990F8A}" name="Tabla1" displayName="Tabla1" ref="A1:BW121" totalsRowShown="0" headerRowDxfId="3" headerRowBorderDxfId="2" tableBorderDxfId="1">
+  <autoFilter ref="A1:BW121" xr:uid="{3111F1FF-B489-4444-B033-EAAA6A990F8A}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:BW100">
     <sortCondition descending="1" ref="AK1:AK100"/>
   </sortState>
@@ -10917,7 +11243,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BW117"/>
+  <dimension ref="A1:BW121"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:75" x14ac:dyDescent="0.3">
@@ -37093,6 +37419,902 @@
       </c>
       <c r="BW117">
         <v>2.75655493797955E-3</v>
+      </c>
+    </row>
+    <row r="118" spans="1:75" x14ac:dyDescent="0.3">
+      <c r="A118" s="2">
+        <v>46084.57675925926</v>
+      </c>
+      <c r="B118" t="s">
+        <v>267</v>
+      </c>
+      <c r="C118">
+        <v>3</v>
+      </c>
+      <c r="D118" t="s">
+        <v>76</v>
+      </c>
+      <c r="E118" t="s">
+        <v>77</v>
+      </c>
+      <c r="F118">
+        <v>16590</v>
+      </c>
+      <c r="G118">
+        <v>4.5</v>
+      </c>
+      <c r="H118" t="s">
+        <v>171</v>
+      </c>
+      <c r="I118" t="s">
+        <v>79</v>
+      </c>
+      <c r="J118">
+        <v>5</v>
+      </c>
+      <c r="K118">
+        <v>5</v>
+      </c>
+      <c r="L118" t="s">
+        <v>80</v>
+      </c>
+      <c r="M118" t="s">
+        <v>81</v>
+      </c>
+      <c r="N118" t="s">
+        <v>82</v>
+      </c>
+      <c r="O118" t="s">
+        <v>82</v>
+      </c>
+      <c r="P118" t="s">
+        <v>83</v>
+      </c>
+      <c r="Q118" t="s">
+        <v>265</v>
+      </c>
+      <c r="R118">
+        <v>4</v>
+      </c>
+      <c r="S118" t="s">
+        <v>85</v>
+      </c>
+      <c r="T118" t="s">
+        <v>86</v>
+      </c>
+      <c r="U118" t="s">
+        <v>108</v>
+      </c>
+      <c r="V118">
+        <v>2</v>
+      </c>
+      <c r="W118" t="s">
+        <v>173</v>
+      </c>
+      <c r="X118" t="s">
+        <v>82</v>
+      </c>
+      <c r="Y118" t="s">
+        <v>89</v>
+      </c>
+      <c r="Z118">
+        <v>4000</v>
+      </c>
+      <c r="AA118">
+        <v>4000</v>
+      </c>
+      <c r="AC118">
+        <v>512</v>
+      </c>
+      <c r="AD118" t="s">
+        <v>90</v>
+      </c>
+      <c r="AE118">
+        <v>0.1</v>
+      </c>
+      <c r="AF118">
+        <v>200</v>
+      </c>
+      <c r="AG118">
+        <v>80</v>
+      </c>
+      <c r="AH118">
+        <v>120</v>
+      </c>
+      <c r="AI118">
+        <v>8.1052205736362792E-2</v>
+      </c>
+      <c r="AJ118">
+        <v>14.22849995965816</v>
+      </c>
+      <c r="AK118">
+        <v>0.77746501612623886</v>
+      </c>
+      <c r="AL118">
+        <v>-0.3388975246539947</v>
+      </c>
+      <c r="AM118">
+        <v>15.862007738386041</v>
+      </c>
+      <c r="AN118">
+        <v>0.78442861878483838</v>
+      </c>
+      <c r="AO118">
+        <v>15.862007738386041</v>
+      </c>
+      <c r="AP118">
+        <v>15.862007738386041</v>
+      </c>
+      <c r="AQ118">
+        <v>0.78442861878483838</v>
+      </c>
+      <c r="AR118">
+        <v>121.20113997537661</v>
+      </c>
+      <c r="AS118">
+        <v>-8.1210961546633792E-2</v>
+      </c>
+      <c r="AT118">
+        <v>0.8</v>
+      </c>
+      <c r="AU118" t="s">
+        <v>91</v>
+      </c>
+      <c r="AV118">
+        <v>2.8301968546252301E-2</v>
+      </c>
+      <c r="AW118">
+        <v>0.79449111508239822</v>
+      </c>
+      <c r="AX118">
+        <v>2.8301968546252301E-2</v>
+      </c>
+      <c r="AY118">
+        <v>2.8301968546252301E-2</v>
+      </c>
+      <c r="AZ118">
+        <v>0.79449111508239822</v>
+      </c>
+      <c r="BA118">
+        <v>8.7375441623793029E-2</v>
+      </c>
+      <c r="BB118">
+        <v>0.36554132098820119</v>
+      </c>
+      <c r="BC118">
+        <v>8.5353100083140371E-2</v>
+      </c>
+      <c r="BD118">
+        <v>0.70426973809866467</v>
+      </c>
+      <c r="BE118">
+        <v>8.5353100083140371E-2</v>
+      </c>
+      <c r="BF118">
+        <v>8.5353100083140371E-2</v>
+      </c>
+      <c r="BG118">
+        <v>0.70426973809866467</v>
+      </c>
+      <c r="BH118">
+        <v>0.25345929775810411</v>
+      </c>
+      <c r="BI118">
+        <v>0.12181766761464741</v>
+      </c>
+      <c r="BJ118">
+        <v>4.5063036259409023E-2</v>
+      </c>
+      <c r="BK118">
+        <v>0.81908616294267955</v>
+      </c>
+      <c r="BL118">
+        <v>4.5063036259409023E-2</v>
+      </c>
+      <c r="BM118">
+        <v>4.5063036259409023E-2</v>
+      </c>
+      <c r="BN118">
+        <v>0.81908616294267955</v>
+      </c>
+      <c r="BO118">
+        <v>0.35727610205897897</v>
+      </c>
+      <c r="BP118">
+        <v>-0.43435054265516498</v>
+      </c>
+      <c r="BQ118">
+        <v>63.289312848655371</v>
+      </c>
+      <c r="BR118">
+        <v>0.81986745901560942</v>
+      </c>
+      <c r="BS118">
+        <v>63.289312848655371</v>
+      </c>
+      <c r="BT118">
+        <v>63.289312848655371</v>
+      </c>
+      <c r="BU118">
+        <v>0.81986745901560942</v>
+      </c>
+      <c r="BV118">
+        <v>484.10644906006519</v>
+      </c>
+      <c r="BW118">
+        <v>-0.37785229213422711</v>
+      </c>
+    </row>
+    <row r="119" spans="1:75" x14ac:dyDescent="0.3">
+      <c r="A119" s="2">
+        <v>46084.906828703701</v>
+      </c>
+      <c r="B119" t="s">
+        <v>268</v>
+      </c>
+      <c r="C119">
+        <v>1</v>
+      </c>
+      <c r="D119" t="s">
+        <v>76</v>
+      </c>
+      <c r="E119" t="s">
+        <v>77</v>
+      </c>
+      <c r="F119">
+        <v>16590</v>
+      </c>
+      <c r="G119">
+        <v>4.5</v>
+      </c>
+      <c r="H119" t="s">
+        <v>171</v>
+      </c>
+      <c r="I119" t="s">
+        <v>79</v>
+      </c>
+      <c r="J119">
+        <v>5</v>
+      </c>
+      <c r="K119">
+        <v>5</v>
+      </c>
+      <c r="L119" t="s">
+        <v>80</v>
+      </c>
+      <c r="M119" t="s">
+        <v>81</v>
+      </c>
+      <c r="N119" t="s">
+        <v>82</v>
+      </c>
+      <c r="O119" t="s">
+        <v>82</v>
+      </c>
+      <c r="P119" t="s">
+        <v>83</v>
+      </c>
+      <c r="Q119" t="s">
+        <v>269</v>
+      </c>
+      <c r="R119">
+        <v>4</v>
+      </c>
+      <c r="S119" t="s">
+        <v>85</v>
+      </c>
+      <c r="T119" t="s">
+        <v>86</v>
+      </c>
+      <c r="U119" t="s">
+        <v>108</v>
+      </c>
+      <c r="V119">
+        <v>3</v>
+      </c>
+      <c r="W119" t="s">
+        <v>173</v>
+      </c>
+      <c r="X119" t="s">
+        <v>82</v>
+      </c>
+      <c r="Y119" t="s">
+        <v>89</v>
+      </c>
+      <c r="Z119">
+        <v>4000</v>
+      </c>
+      <c r="AA119">
+        <v>4000</v>
+      </c>
+      <c r="AC119">
+        <v>512</v>
+      </c>
+      <c r="AD119" t="s">
+        <v>90</v>
+      </c>
+      <c r="AE119">
+        <v>0.1</v>
+      </c>
+      <c r="AF119">
+        <v>240</v>
+      </c>
+      <c r="AG119">
+        <v>120</v>
+      </c>
+      <c r="AH119">
+        <v>120</v>
+      </c>
+      <c r="AI119">
+        <v>0.106008494446163</v>
+      </c>
+      <c r="AJ119">
+        <v>33.838931129888543</v>
+      </c>
+      <c r="AK119">
+        <v>0.66621549860948348</v>
+      </c>
+      <c r="AL119">
+        <v>5.3792376803492359E-2</v>
+      </c>
+      <c r="AM119">
+        <v>35.082387455197612</v>
+      </c>
+      <c r="AN119">
+        <v>0.68480606442805336</v>
+      </c>
+      <c r="AO119">
+        <v>35.082387455197612</v>
+      </c>
+      <c r="AP119">
+        <v>35.082387455197612</v>
+      </c>
+      <c r="AQ119">
+        <v>0.68480606442805336</v>
+      </c>
+      <c r="AR119">
+        <v>114.439596298278</v>
+      </c>
+      <c r="AS119">
+        <v>-0.61720424299988363</v>
+      </c>
+      <c r="AT119">
+        <v>0.8</v>
+      </c>
+      <c r="AU119" t="s">
+        <v>91</v>
+      </c>
+      <c r="AV119">
+        <v>3.8320129051456348E-2</v>
+      </c>
+      <c r="AW119">
+        <v>0.72174631674847922</v>
+      </c>
+      <c r="AX119">
+        <v>3.8320129051456348E-2</v>
+      </c>
+      <c r="AY119">
+        <v>3.8320129051456348E-2</v>
+      </c>
+      <c r="AZ119">
+        <v>0.72174631674847922</v>
+      </c>
+      <c r="BA119">
+        <v>0.1118626898969249</v>
+      </c>
+      <c r="BB119">
+        <v>0.1877322375285925</v>
+      </c>
+      <c r="BC119">
+        <v>8.0002391425953584E-2</v>
+      </c>
+      <c r="BD119">
+        <v>0.72280880078070253</v>
+      </c>
+      <c r="BE119">
+        <v>8.0002391425953584E-2</v>
+      </c>
+      <c r="BF119">
+        <v>8.0002391425953584E-2</v>
+      </c>
+      <c r="BG119">
+        <v>0.72280880078070253</v>
+      </c>
+      <c r="BH119">
+        <v>0.3205165810134426</v>
+      </c>
+      <c r="BI119">
+        <v>-0.1105214966357024</v>
+      </c>
+      <c r="BJ119">
+        <v>7.6340327560767682E-2</v>
+      </c>
+      <c r="BK119">
+        <v>0.69351773143454143</v>
+      </c>
+      <c r="BL119">
+        <v>7.6340327560767682E-2</v>
+      </c>
+      <c r="BM119">
+        <v>7.6340327560767682E-2</v>
+      </c>
+      <c r="BN119">
+        <v>0.69351773143454143</v>
+      </c>
+      <c r="BO119">
+        <v>0.80870605181118038</v>
+      </c>
+      <c r="BP119">
+        <v>-2.2466990027572451</v>
+      </c>
+      <c r="BQ119">
+        <v>140.13488697275301</v>
+      </c>
+      <c r="BR119">
+        <v>0.6011514087484886</v>
+      </c>
+      <c r="BS119">
+        <v>140.13488697275301</v>
+      </c>
+      <c r="BT119">
+        <v>140.13488697275301</v>
+      </c>
+      <c r="BU119">
+        <v>0.6011514087484886</v>
+      </c>
+      <c r="BV119">
+        <v>456.51729987039209</v>
+      </c>
+      <c r="BW119">
+        <v>-0.29932871013520312</v>
+      </c>
+    </row>
+    <row r="120" spans="1:75" x14ac:dyDescent="0.3">
+      <c r="A120" s="2">
+        <v>46085.222731481481</v>
+      </c>
+      <c r="B120" t="s">
+        <v>270</v>
+      </c>
+      <c r="C120">
+        <v>2</v>
+      </c>
+      <c r="D120" t="s">
+        <v>76</v>
+      </c>
+      <c r="E120" t="s">
+        <v>77</v>
+      </c>
+      <c r="F120">
+        <v>16590</v>
+      </c>
+      <c r="G120">
+        <v>4.5</v>
+      </c>
+      <c r="H120" t="s">
+        <v>171</v>
+      </c>
+      <c r="I120" t="s">
+        <v>79</v>
+      </c>
+      <c r="J120">
+        <v>5</v>
+      </c>
+      <c r="K120">
+        <v>5</v>
+      </c>
+      <c r="L120" t="s">
+        <v>80</v>
+      </c>
+      <c r="M120" t="s">
+        <v>81</v>
+      </c>
+      <c r="N120" t="s">
+        <v>82</v>
+      </c>
+      <c r="O120" t="s">
+        <v>82</v>
+      </c>
+      <c r="P120" t="s">
+        <v>83</v>
+      </c>
+      <c r="Q120" t="s">
+        <v>269</v>
+      </c>
+      <c r="R120">
+        <v>4</v>
+      </c>
+      <c r="S120" t="s">
+        <v>85</v>
+      </c>
+      <c r="T120" t="s">
+        <v>86</v>
+      </c>
+      <c r="U120" t="s">
+        <v>108</v>
+      </c>
+      <c r="V120">
+        <v>3</v>
+      </c>
+      <c r="W120" t="s">
+        <v>173</v>
+      </c>
+      <c r="X120" t="s">
+        <v>82</v>
+      </c>
+      <c r="Y120" t="s">
+        <v>89</v>
+      </c>
+      <c r="Z120">
+        <v>4000</v>
+      </c>
+      <c r="AA120">
+        <v>4000</v>
+      </c>
+      <c r="AC120">
+        <v>512</v>
+      </c>
+      <c r="AD120" t="s">
+        <v>90</v>
+      </c>
+      <c r="AE120">
+        <v>0.1</v>
+      </c>
+      <c r="AF120">
+        <v>240</v>
+      </c>
+      <c r="AG120">
+        <v>120</v>
+      </c>
+      <c r="AH120">
+        <v>120</v>
+      </c>
+      <c r="AI120">
+        <v>8.6326044526204557E-2</v>
+      </c>
+      <c r="AJ120">
+        <v>14.146799722733681</v>
+      </c>
+      <c r="AK120">
+        <v>0.72262530601792541</v>
+      </c>
+      <c r="AL120">
+        <v>7.581434566459494E-2</v>
+      </c>
+      <c r="AM120">
+        <v>25.026228384313718</v>
+      </c>
+      <c r="AN120">
+        <v>0.73291761438861314</v>
+      </c>
+      <c r="AO120">
+        <v>25.026228384313718</v>
+      </c>
+      <c r="AP120">
+        <v>25.026228384313718</v>
+      </c>
+      <c r="AQ120">
+        <v>0.73291761438861314</v>
+      </c>
+      <c r="AR120">
+        <v>120.5007286916416</v>
+      </c>
+      <c r="AS120">
+        <v>4.6809187335239033E-2</v>
+      </c>
+      <c r="AT120">
+        <v>0.8</v>
+      </c>
+      <c r="AU120" t="s">
+        <v>91</v>
+      </c>
+      <c r="AV120">
+        <v>4.3604468438270379E-2</v>
+      </c>
+      <c r="AW120">
+        <v>0.68337518036849354</v>
+      </c>
+      <c r="AX120">
+        <v>4.3604468438270379E-2</v>
+      </c>
+      <c r="AY120">
+        <v>4.3604468438270379E-2</v>
+      </c>
+      <c r="AZ120">
+        <v>0.68337518036849354</v>
+      </c>
+      <c r="BA120">
+        <v>0.15250768795884201</v>
+      </c>
+      <c r="BB120">
+        <v>-0.10740300069810479</v>
+      </c>
+      <c r="BC120">
+        <v>0.10193258953106291</v>
+      </c>
+      <c r="BD120">
+        <v>0.64682534824230808</v>
+      </c>
+      <c r="BE120">
+        <v>0.10193258953106291</v>
+      </c>
+      <c r="BF120">
+        <v>0.10193258953106291</v>
+      </c>
+      <c r="BG120">
+        <v>0.64682534824230808</v>
+      </c>
+      <c r="BH120">
+        <v>0.30160015428650921</v>
+      </c>
+      <c r="BI120">
+        <v>-4.4980118235335993E-2</v>
+      </c>
+      <c r="BJ120">
+        <v>2.8422902017742321E-2</v>
+      </c>
+      <c r="BK120">
+        <v>0.88589103861681395</v>
+      </c>
+      <c r="BL120">
+        <v>2.8422902017742321E-2</v>
+      </c>
+      <c r="BM120">
+        <v>2.8422902017742321E-2</v>
+      </c>
+      <c r="BN120">
+        <v>0.88589103861681395</v>
+      </c>
+      <c r="BO120">
+        <v>7.2238055104180895E-2</v>
+      </c>
+      <c r="BP120">
+        <v>0.70998705779114513</v>
+      </c>
+      <c r="BQ120">
+        <v>99.930953577267957</v>
+      </c>
+      <c r="BR120">
+        <v>0.7155788903268383</v>
+      </c>
+      <c r="BS120">
+        <v>99.930953577267957</v>
+      </c>
+      <c r="BT120">
+        <v>99.930953577267957</v>
+      </c>
+      <c r="BU120">
+        <v>0.7155788903268383</v>
+      </c>
+      <c r="BV120">
+        <v>481.47656886921482</v>
+      </c>
+      <c r="BW120">
+        <v>-0.37036718951674041</v>
+      </c>
+    </row>
+    <row r="121" spans="1:75" x14ac:dyDescent="0.3">
+      <c r="A121" s="2">
+        <v>46085.564212962963</v>
+      </c>
+      <c r="B121" t="s">
+        <v>271</v>
+      </c>
+      <c r="C121">
+        <v>3</v>
+      </c>
+      <c r="D121" t="s">
+        <v>101</v>
+      </c>
+      <c r="E121" t="s">
+        <v>77</v>
+      </c>
+      <c r="F121">
+        <v>16590</v>
+      </c>
+      <c r="G121">
+        <v>4.5</v>
+      </c>
+      <c r="H121" t="s">
+        <v>171</v>
+      </c>
+      <c r="I121" t="s">
+        <v>79</v>
+      </c>
+      <c r="J121">
+        <v>5</v>
+      </c>
+      <c r="K121">
+        <v>5</v>
+      </c>
+      <c r="L121" t="s">
+        <v>80</v>
+      </c>
+      <c r="M121" t="s">
+        <v>81</v>
+      </c>
+      <c r="N121" t="s">
+        <v>82</v>
+      </c>
+      <c r="O121" t="s">
+        <v>82</v>
+      </c>
+      <c r="P121" t="s">
+        <v>83</v>
+      </c>
+      <c r="Q121" t="s">
+        <v>269</v>
+      </c>
+      <c r="R121">
+        <v>4</v>
+      </c>
+      <c r="S121" t="s">
+        <v>85</v>
+      </c>
+      <c r="T121" t="s">
+        <v>86</v>
+      </c>
+      <c r="U121" t="s">
+        <v>108</v>
+      </c>
+      <c r="V121">
+        <v>3</v>
+      </c>
+      <c r="W121" t="s">
+        <v>173</v>
+      </c>
+      <c r="X121" t="s">
+        <v>82</v>
+      </c>
+      <c r="Y121" t="s">
+        <v>89</v>
+      </c>
+      <c r="Z121">
+        <v>4000</v>
+      </c>
+      <c r="AA121">
+        <v>4000</v>
+      </c>
+      <c r="AC121">
+        <v>512</v>
+      </c>
+      <c r="AD121" t="s">
+        <v>90</v>
+      </c>
+      <c r="AE121">
+        <v>0.1</v>
+      </c>
+      <c r="AF121">
+        <v>240</v>
+      </c>
+      <c r="AG121">
+        <v>120</v>
+      </c>
+      <c r="AH121">
+        <v>120</v>
+      </c>
+      <c r="AI121">
+        <v>0.10290996228240711</v>
+      </c>
+      <c r="AJ121">
+        <v>26.931966029656579</v>
+      </c>
+      <c r="AK121">
+        <v>0.68443970848741087</v>
+      </c>
+      <c r="AL121">
+        <v>8.6293657915927025E-2</v>
+      </c>
+      <c r="AM121">
+        <v>28.812146797667111</v>
+      </c>
+      <c r="AN121">
+        <v>0.67734594458609443</v>
+      </c>
+      <c r="AO121">
+        <v>28.812146797667111</v>
+      </c>
+      <c r="AP121">
+        <v>28.812146797667111</v>
+      </c>
+      <c r="AQ121">
+        <v>0.67734594458609443</v>
+      </c>
+      <c r="AR121">
+        <v>112.7319246644321</v>
+      </c>
+      <c r="AS121">
+        <v>1.2595647239736749E-2</v>
+      </c>
+      <c r="AT121">
+        <v>0.8</v>
+      </c>
+      <c r="AU121" t="s">
+        <v>91</v>
+      </c>
+      <c r="AV121">
+        <v>3.4941550989431677E-2</v>
+      </c>
+      <c r="AW121">
+        <v>0.74627916184012233</v>
+      </c>
+      <c r="AX121">
+        <v>3.4941550989431677E-2</v>
+      </c>
+      <c r="AY121">
+        <v>3.4941550989431677E-2</v>
+      </c>
+      <c r="AZ121">
+        <v>0.74627916184012233</v>
+      </c>
+      <c r="BA121">
+        <v>0.1223043357798201</v>
+      </c>
+      <c r="BB121">
+        <v>0.1119123878036022</v>
+      </c>
+      <c r="BC121">
+        <v>0.1088797158354875</v>
+      </c>
+      <c r="BD121">
+        <v>0.62275503937868226</v>
+      </c>
+      <c r="BE121">
+        <v>0.1088797158354875</v>
+      </c>
+      <c r="BF121">
+        <v>0.1088797158354875</v>
+      </c>
+      <c r="BG121">
+        <v>0.62275503937868226</v>
+      </c>
+      <c r="BH121">
+        <v>0.26707186033242392</v>
+      </c>
+      <c r="BI121">
+        <v>7.465304569311626E-2</v>
+      </c>
+      <c r="BJ121">
+        <v>8.2765557334563297E-2</v>
+      </c>
+      <c r="BK121">
+        <v>0.66772246620516862</v>
+      </c>
+      <c r="BL121">
+        <v>8.2765557334563297E-2</v>
+      </c>
+      <c r="BM121">
+        <v>8.2765557334563297E-2</v>
+      </c>
+      <c r="BN121">
+        <v>0.66772246620516862</v>
+      </c>
+      <c r="BO121">
+        <v>0.21283797098879029</v>
+      </c>
+      <c r="BP121">
+        <v>0.14552286753565319</v>
+      </c>
+      <c r="BQ121">
+        <v>115.0220003665092</v>
+      </c>
+      <c r="BR121">
+        <v>0.6726271109204025</v>
+      </c>
+      <c r="BS121">
+        <v>115.0220003665092</v>
+      </c>
+      <c r="BT121">
+        <v>115.0220003665092</v>
+      </c>
+      <c r="BU121">
+        <v>0.6726271109204025</v>
+      </c>
+      <c r="BV121">
+        <v>450.32548449062648</v>
+      </c>
+      <c r="BW121">
+        <v>-0.28170571207342049</v>
       </c>
     </row>
   </sheetData>
@@ -37105,7 +38327,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC2417C5-69B1-40A5-8AFE-A835A2C478FA}">
-  <dimension ref="A2:L67"/>
+  <dimension ref="A2:L68"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="41.21875" bestFit="1" customWidth="1"/>
@@ -39217,37 +40439,37 @@
         <v>4</v>
       </c>
       <c r="B57" s="9">
-        <v>0.75718351490092817</v>
+        <v>0.74729526321411399</v>
       </c>
       <c r="C57" s="9">
-        <v>9.0357583941765449E-2</v>
+        <v>6.3444946161929791E-2</v>
       </c>
       <c r="D57" s="9">
-        <v>0.68237250738338795</v>
+        <v>0.69439482652260698</v>
       </c>
       <c r="E57" s="9">
-        <v>0.75559966964583858</v>
+        <v>0.73750301675233876</v>
       </c>
       <c r="F57" s="9">
-        <v>0.7691136920645919</v>
+        <v>0.76854494933908279</v>
       </c>
       <c r="G57" s="9">
-        <v>0.74813842536074693</v>
+        <v>0.73795349022565537</v>
       </c>
       <c r="H57" s="9">
-        <v>0.1345855381242079</v>
+        <v>0.13566558218673344</v>
       </c>
       <c r="I57" s="9">
-        <v>8.8923566883683441E-2</v>
+        <v>7.143883526712741E-2</v>
       </c>
       <c r="J57" s="9">
-        <v>0.3307414800923682</v>
+        <v>0.15582450562264127</v>
       </c>
       <c r="K57" s="9">
-        <v>-0.15751719749678442</v>
+        <v>-0.19636081493414295</v>
       </c>
       <c r="L57" s="9">
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.3">
@@ -39483,37 +40705,37 @@
         <v>108</v>
       </c>
       <c r="B64" s="9">
-        <v>0.79986929126743034</v>
+        <v>0.74174735196265329</v>
       </c>
       <c r="C64" s="9">
-        <v>0.12098667290639745</v>
+        <v>1.9829366923802421E-2</v>
       </c>
       <c r="D64" s="9">
-        <v>0.84901952677310621</v>
+        <v>0.77398847126428427</v>
       </c>
       <c r="E64" s="9">
-        <v>0.75043565674835844</v>
+        <v>0.69958837333284574</v>
       </c>
       <c r="F64" s="9">
-        <v>0.78575563806377979</v>
+        <v>0.77295477922112721</v>
       </c>
       <c r="G64" s="9">
-        <v>0.8153458995874403</v>
+        <v>0.73998611136436987</v>
       </c>
       <c r="H64" s="9">
-        <v>0.57687824796147791</v>
+        <v>0.28525657359087447</v>
       </c>
       <c r="I64" s="9">
-        <v>8.955955391420839E-2</v>
+        <v>3.6681367710857005E-2</v>
       </c>
       <c r="J64" s="9">
-        <v>0.48293696159763283</v>
+        <v>-0.14327761614839099</v>
       </c>
       <c r="K64" s="9">
-        <v>-0.79824197526474627</v>
+        <v>-0.48762297573151397</v>
       </c>
       <c r="L64" s="9">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.3">
@@ -39521,113 +40743,151 @@
         <v>86</v>
       </c>
       <c r="B65" s="9">
-        <v>0.79986929126743034</v>
+        <v>0.74174735196265329</v>
       </c>
       <c r="C65" s="9">
-        <v>0.12098667290639745</v>
+        <v>1.9829366923802421E-2</v>
       </c>
       <c r="D65" s="9">
-        <v>0.84901952677310621</v>
+        <v>0.77398847126428427</v>
       </c>
       <c r="E65" s="9">
-        <v>0.75043565674835844</v>
+        <v>0.69958837333284574</v>
       </c>
       <c r="F65" s="9">
-        <v>0.78575563806377979</v>
+        <v>0.77295477922112721</v>
       </c>
       <c r="G65" s="9">
-        <v>0.8153458995874403</v>
+        <v>0.73998611136436987</v>
       </c>
       <c r="H65" s="9">
-        <v>0.57687824796147791</v>
+        <v>0.28525657359087447</v>
       </c>
       <c r="I65" s="9">
-        <v>8.955955391420839E-2</v>
+        <v>3.6681367710857005E-2</v>
       </c>
       <c r="J65" s="9">
-        <v>0.48293696159763283</v>
+        <v>-0.14327761614839099</v>
       </c>
       <c r="K65" s="9">
-        <v>-0.79824197526474627</v>
+        <v>-0.48762297573151397</v>
       </c>
       <c r="L65" s="9">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A66" s="8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B66" s="9">
-        <v>0.79986929126743034</v>
+        <v>0.69109350437160655</v>
       </c>
       <c r="C66" s="9">
-        <v>0.12098667290639745</v>
+        <v>7.1966793461338108E-2</v>
       </c>
       <c r="D66" s="9">
-        <v>0.84901952677310621</v>
+        <v>0.71713355298569825</v>
       </c>
       <c r="E66" s="9">
-        <v>0.75043565674835844</v>
+        <v>0.66412972946723092</v>
       </c>
       <c r="F66" s="9">
-        <v>0.78575563806377979</v>
+        <v>0.74904374541884133</v>
       </c>
       <c r="G66" s="9">
-        <v>0.8153458995874403</v>
+        <v>0.66311913666524314</v>
       </c>
       <c r="H66" s="9">
-        <v>0.57687824796147791</v>
+        <v>6.4080541544696626E-2</v>
       </c>
       <c r="I66" s="9">
-        <v>8.955955391420839E-2</v>
+        <v>-2.6949523059307378E-2</v>
       </c>
       <c r="J66" s="9">
-        <v>0.48293696159763283</v>
+        <v>-0.46372969247681556</v>
       </c>
       <c r="K66" s="9">
-        <v>-0.79824197526474627</v>
+        <v>-0.31713387057512138</v>
       </c>
       <c r="L66" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A67" s="3" t="s">
+      <c r="A67" s="8">
+        <v>2</v>
+      </c>
+      <c r="B67" s="9">
+        <v>0.79240119955369981</v>
+      </c>
+      <c r="C67" s="9">
+        <v>-3.2308059613733266E-2</v>
+      </c>
+      <c r="D67" s="9">
+        <v>0.83084338954287018</v>
+      </c>
+      <c r="E67" s="9">
+        <v>0.73504701719846055</v>
+      </c>
+      <c r="F67" s="9">
+        <v>0.79686581302341308</v>
+      </c>
+      <c r="G67" s="9">
+        <v>0.81685308606349671</v>
+      </c>
+      <c r="H67" s="9">
+        <v>0.50643260563705239</v>
+      </c>
+      <c r="I67" s="9">
+        <v>0.10031225848102139</v>
+      </c>
+      <c r="J67" s="9">
+        <v>0.17717446018003358</v>
+      </c>
+      <c r="K67" s="9">
+        <v>-0.65811208088790651</v>
+      </c>
+      <c r="L67" s="9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A68" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="B67" s="9">
-        <v>0.6000573113155343</v>
-      </c>
-      <c r="C67" s="9">
-        <v>-7.3687783208431154E-2</v>
-      </c>
-      <c r="D67" s="9">
-        <v>0.43954667678608356</v>
-      </c>
-      <c r="E67" s="9">
-        <v>0.63567473010720454</v>
-      </c>
-      <c r="F67" s="9">
-        <v>0.52406824138797692</v>
-      </c>
-      <c r="G67" s="9">
-        <v>0.70166207335070352</v>
-      </c>
-      <c r="H67" s="9">
-        <v>-0.10978850568749605</v>
-      </c>
-      <c r="I67" s="9">
-        <v>7.5616782188577758E-2</v>
-      </c>
-      <c r="J67" s="9">
-        <v>0.14440727588182414</v>
-      </c>
-      <c r="K67" s="9">
-        <v>-0.21806963769529558</v>
-      </c>
-      <c r="L67" s="9">
-        <v>116</v>
+      <c r="B68" s="9">
+        <v>0.60381161368202541</v>
+      </c>
+      <c r="C68" s="9">
+        <v>-7.2256499970399929E-2</v>
+      </c>
+      <c r="D68" s="9">
+        <v>0.44944421901020987</v>
+      </c>
+      <c r="E68" s="9">
+        <v>0.63695773015780055</v>
+      </c>
+      <c r="F68" s="9">
+        <v>0.53215111166837104</v>
+      </c>
+      <c r="G68" s="9">
+        <v>0.70168354481410788</v>
+      </c>
+      <c r="H68" s="9">
+        <v>-0.10148069761772709</v>
+      </c>
+      <c r="I68" s="9">
+        <v>7.3437631935931211E-2</v>
+      </c>
+      <c r="J68" s="9">
+        <v>0.12438086985171655</v>
+      </c>
+      <c r="K68" s="9">
+        <v>-0.22187776563761569</v>
+      </c>
+      <c r="L68" s="9">
+        <v>120</v>
       </c>
     </row>
   </sheetData>

</xml_diff>